<commit_message>
Further improvements to output
</commit_message>
<xml_diff>
--- a/outputs/botecs/rheumatic_heart_disease_prevention.xlsx
+++ b/outputs/botecs/rheumatic_heart_disease_prevention.xlsx
@@ -182,6 +182,12 @@
 https://www.ahajournals.org/doi/10.1161/circ.150.suppl_1.4144731</t>
       </text>
     </comment>
+    <comment ref="C20" authorId="0" shapeId="0">
+      <text>
+        <t>The original QEA stated: "I am concerned that the cost estimate (from the academic lit) may be an underestimate, possibly a gross one." and noted the intervention would still be 10x cash at 6x cost increase.
+https://docs.google.com/document/d/1siZVFAA3E3SLWroQ_oQqTuxUBMfEYvM_z8tL6eOp2Y8/edit</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -475,10 +481,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
   </cols>
@@ -486,7 +492,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Mortality benefit</t>
+          <t>Burden &amp; effect</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -518,7 +524,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Internal validity adjustment</t>
+          <t>Internal validity (IV) adjustment</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
@@ -533,7 +539,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>External validity adjustment</t>
+          <t>External validity (EV) adjustment</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
@@ -609,160 +615,144 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Units of value per RHD death averted (GW moral weights)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>GiveWell moral weights for LMIC adult death. Unchanged.</t>
-        </is>
-      </c>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Mortality benefit</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Total units of value per 100,000 cohort</t>
-        </is>
-      </c>
-      <c r="B10" s="9">
-        <f>B8*B9</f>
-        <v/>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
+          <t>Units of value per RHD death averted (GW moral weights)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>52.5</v>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>GiveWell moral weights for LMIC adult death. Unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>UoV from mortality per 100,000 cohort</t>
+        </is>
+      </c>
+      <c r="B11" s="9">
+        <f>B8*B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Calculation</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Costs</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="n"/>
-    </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Annual program cost in 2010 USD (Watkins et al. 2015)</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n">
-        <v>20289</v>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>From Cuba study. No new cost data found. GiveWell considered this 'possibly a gross underestimate'.</t>
-        </is>
-      </c>
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Ad-hoc benefit adjustments (subjective)</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CPI inflation factor (2010 → 2026)</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>I'm estimating ~1.46 for 2010→2026. Should verify with BLS CPI calculator.</t>
+          <t>Morbidity uplift: YLDs averted from RHD (% of mortality UoV)</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>I'm assuming +30%. RHD causes chronic heart failure, reduced exercise tolerance, and need for lifelong secondary prophylaxis. This is a rough guess — not verified against GBD YLD data.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Annual program cost in 2026 USD</t>
-        </is>
-      </c>
-      <c r="B14" s="11">
-        <f>B12*B13</f>
-        <v/>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Calculation</t>
+          <t>Perinatal outcomes uplift (% of mortality UoV)</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>I'm assuming +15%. RHD is 'the principal heart disease seen in pregnant women' per WHO; causes maternal and perinatal morbidity/mortality. Rough guess.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Number covered by program annually (Watkins et al. 2015)</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>273933</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>From original Cuba study</t>
+          <t>Total UoV per 100,000 cohort (with adjustments)</t>
+        </is>
+      </c>
+      <c r="B15" s="9">
+        <f>B11*(1+B13+B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>Calculation: mortality UoV x (1 + morbidity + perinatal)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Annual cost per beneficiary</t>
-        </is>
-      </c>
-      <c r="B16" s="12">
-        <f>B14/B15</f>
-        <v/>
-      </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Calculation</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Duration of intervention per beneficiary (years)</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>19</v>
-      </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Covers ages 5-24. Unchanged from original.</t>
+          <t>Annual program cost in 2010 USD (Watkins et al. 2015)</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>20289</v>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>From Cuba study. No new cost data found. GiveWell considered this 'possibly a gross underestimate'.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Total cost per beneficiary (lifetime)</t>
-        </is>
-      </c>
-      <c r="B18" s="12">
-        <f>B16*B17</f>
-        <v/>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Calculation</t>
+          <t>CPI inflation factor (2010 → 2026)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>I'm estimating ~1.46 for 2010→2026. Should verify with BLS CPI calculator.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Total cost per 100,000 cohort</t>
+          <t>Annual program cost in 2026 USD (pre-adjustment)</t>
         </is>
       </c>
       <c r="B19" s="11">
-        <f>B18*100000</f>
+        <f>B17*B18</f>
         <v/>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -772,21 +762,28 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Final CE estimate</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Subjective cost multiplier</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>I'm assuming 3x. Cuba has universal free healthcare with existing primary care infrastructure; India would need to build screening, treatment, and referral systems. 3x is moderate — at 5x the CE is still ~16x (above bar). At 1x (original) CE is ~54x (almost certainly too high).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Units of value per $100,000 donated</t>
-        </is>
-      </c>
-      <c r="B21" s="9">
-        <f>B10/B19*100000</f>
+          <t>Adjusted annual program cost in 2026 USD</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>B19*B20</f>
         <v/>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -798,26 +795,26 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>GiveDirectly units of value per $100,000</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>344</v>
+          <t>Number covered by program annually (Watkins et al. 2015)</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>273933</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>GW benchmark</t>
+          <t>From original Cuba study</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cost per death averted</t>
-        </is>
-      </c>
-      <c r="B23" s="11">
-        <f>B19/B8</f>
+          <t>Adjusted annual cost per beneficiary</t>
+        </is>
+      </c>
+      <c r="B23" s="12">
+        <f>B21/B22</f>
         <v/>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -829,16 +826,118 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Duration of intervention per beneficiary (years)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>19</v>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Covers ages 5-24. Unchanged from original.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Total cost per beneficiary (lifetime)</t>
+        </is>
+      </c>
+      <c r="B25" s="12">
+        <f>B23*B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Total cost per 100,000 cohort</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>B25*100000</f>
+        <v/>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>Final CE estimate</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Units of value per $100,000 donated</t>
+        </is>
+      </c>
+      <c r="B28" s="9">
+        <f>B15/B26*100000</f>
+        <v/>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GiveDirectly units of value per $100,000</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>344</v>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>GW benchmark</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Cost per death averted</t>
+        </is>
+      </c>
+      <c r="B30" s="11">
+        <f>B26/B8</f>
+        <v/>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Calculation (mortality only; does not include morbidity/perinatal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>CE (multiples of cash)</t>
         </is>
       </c>
-      <c r="B24" s="13">
-        <f>B21/B22</f>
-        <v/>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Main result. Almost certainly overstated due to cost underestimation.</t>
+      <c r="B31" s="13">
+        <f>B28/B29</f>
+        <v/>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>Best-guess estimate. Includes 3x cost multiplier and ad-hoc benefit adjustments. At 5x cost multiplier → ~16x. Confidence: Low (cost is pivotal unknown).</t>
         </is>
       </c>
     </row>
@@ -847,11 +946,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>